<commit_message>
Process the seven full texts the researcher put in the Drive inbox (S015, S037, S104, S142, S270, S294, S388); sticky second-extractor sample; test hardening
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014MhMGnb8qDcM9MkpTmcbeG
</commit_message>
<xml_diff>
--- a/legal-last-mile-systematic-review/03_extraction/second_extractor/second_extractor_sheet_BLANK_2026-10-04.xlsx
+++ b/legal-last-mile-systematic-review/03_extraction/second_extractor/second_extractor_sheet_BLANK_2026-10-04.xlsx
@@ -2508,7 +2508,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Unincorporated status and poverty rate are significantly associated with reduced centralized water/wastewater infrastructure access; sewer coverage rates significantly lower for unincorporated communities near municipal boundaries, consistent with municipal underbounding excluding these areas from service-area expansion.</t>
+          <t>Unincorporated status and poverty rate are significantly associated with reduced centralized water/wastewater infrastructure access; sewer coverage rates significantly lower for unincorporated communities near municipal boundaries, consistent with municipal underbounding excluding these areas from service-area expansion. Full-text check 2026-10-04 (main text; the confidence intervals are in Supple</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr"/>
@@ -4543,7 +4543,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>page 1-2; Abstract: 47% (95% CI 45-49%) overall unavailability rate, provider range 18-76%; OR estimates for h</t>
+          <t>page 1-2; Table 4 p.15 (multilevel logistic regression, n = 3,047, 177 clusters): at least partly owns the hom</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -4593,7 +4593,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>page 1-2; Abstract: 47% (95% CI 45-49%) overall unavailability rate, provider range 18-76%; OR estimates for h</t>
+          <t>page 1-2; Table 4 p.15 (multilevel logistic regression, n = 3,047, 177 clusters): at least partly owns the hom</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>page 1-2; Abstract: 47% (95% CI 45-49%) overall unavailability rate, provider range 18-76%; OR estimates for h</t>
+          <t>page 1-2; Table 4 p.15 (multilevel logistic regression, n = 3,047, 177 clusters): at least partly owns the hom</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>n=3,047 households (2018 DHS), spatially linked to provider data from an international utility database and NWASCO regulator reports</t>
+          <t>n = 3,047 households in 177 household clusters (primary sampling units), 2018 Zambia Demographic and Health Survey, spatially linked to provider data from an international utility database (IBNET) and NWASCO regulator reports; 11 water supply and sanitation companies</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr"/>
@@ -4693,7 +4693,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>page 1-2; Abstract: 47% (95% CI 45-49%) overall unavailability rate, provider range 18-76%; OR estimates for h</t>
+          <t>page 1-2; Table 4 p.15 (multilevel logistic regression, n = 3,047, 177 clusters): at least partly owns the hom</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -4743,7 +4743,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>page 1-2; Abstract: 47% (95% CI 45-49%) overall unavailability rate, provider range 18-76%; OR estimates for h</t>
+          <t>page 1-2; Table 4 p.15 (multilevel logistic regression, n = 3,047, 177 clusters): at least partly owns the hom</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -4793,7 +4793,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>page 1-2; Abstract: 47% (95% CI 45-49%) overall unavailability rate, provider range 18-76%; OR estimates for h</t>
+          <t>page 1-2; Table 4 p.15 (multilevel logistic regression, n = 3,047, 177 clusters): at least partly owns the hom</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -4843,7 +4843,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>page 1-2; Abstract: 47% (95% CI 45-49%) overall unavailability rate, provider range 18-76%; OR estimates for h</t>
+          <t>page 1-2; Table 4 p.15 (multilevel logistic regression, n = 3,047, 177 clusters): at least partly owns the hom</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -4893,7 +4893,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>page 1-2; Abstract: 47% (95% CI 45-49%) overall unavailability rate, provider range 18-76%; OR estimates for h</t>
+          <t>page 1-2; Table 4 p.15 (multilevel logistic regression, n = 3,047, 177 clusters): at least partly owns the hom</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>page 1-2; Abstract: 47% (95% CI 45-49%) overall unavailability rate, provider range 18-76%; OR estimates for h</t>
+          <t>page 1-2; Table 4 p.15 (multilevel logistic regression, n = 3,047, 177 clusters): at least partly owns the hom</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Process third Drive-inbox batch (88 full texts): re-extractions, rechecks, handoff
29 full-text re-extractions, recheck of 15 decided excludes, batch log,
regenerated outputs and counts, handoff/changelog/decision-log updates.
Screening decisions unchanged (A15).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014MhMGnb8qDcM9MkpTmcbeG
</commit_message>
<xml_diff>
--- a/legal-last-mile-systematic-review/03_extraction/second_extractor/second_extractor_sheet_BLANK_2026-10-04.xlsx
+++ b/legal-last-mile-systematic-review/03_extraction/second_extractor/second_extractor_sheet_BLANK_2026-10-04.xlsx
@@ -25807,7 +25807,7 @@
       </c>
       <c r="F515" s="2" t="inlineStr">
         <is>
-          <t>page 169-189; Abstract: households spending &gt;3% of income on water acquisition, DHA vulnerability</t>
+          <t>page 169-189; Method (formulas for average household water spending and the 3% criterion); section on water in Hid</t>
         </is>
       </c>
       <c r="G515" s="2" t="inlineStr">
@@ -25857,7 +25857,7 @@
       </c>
       <c r="F516" s="2" t="inlineStr">
         <is>
-          <t>page 169-189; Abstract: households spending &gt;3% of income on water acquisition, DHA vulnerability</t>
+          <t>page 169-189; Method (formulas for average household water spending and the 3% criterion); section on water in Hid</t>
         </is>
       </c>
       <c r="G516" s="2" t="inlineStr">
@@ -25907,7 +25907,7 @@
       </c>
       <c r="F517" s="2" t="inlineStr">
         <is>
-          <t>page 169-189; Abstract: households spending &gt;3% of income on water acquisition, DHA vulnerability</t>
+          <t>page 169-189; Method (formulas for average household water spending and the 3% criterion); section on water in Hid</t>
         </is>
       </c>
       <c r="G517" s="2" t="inlineStr">
@@ -25922,7 +25922,7 @@
       </c>
       <c r="I517" s="2" t="inlineStr">
         <is>
-          <t>institutional data (national, state, municipal, and water-operator records) analysed to estimate household-level water provision/quality/expenditure proportions</t>
+          <t>84 municipalities of Hidalgo state, Mexico (3,083,841 inhabitants): municipal water tariffs (CAASIM and state official gazette 2022), INEGI household environment module (MOHOMA 2017: mean weekly bottled-water spending of 51.74 pesos, deflated), CONAGUA concession register (REPDA 2022) and the 2020 c</t>
         </is>
       </c>
       <c r="J517" s="2" t="inlineStr"/>
@@ -25957,7 +25957,7 @@
       </c>
       <c r="F518" s="2" t="inlineStr">
         <is>
-          <t>page 169-189; Abstract: households spending &gt;3% of income on water acquisition, DHA vulnerability</t>
+          <t>page 169-189; Method (formulas for average household water spending and the 3% criterion); section on water in Hid</t>
         </is>
       </c>
       <c r="G518" s="2" t="inlineStr">
@@ -26007,7 +26007,7 @@
       </c>
       <c r="F519" s="2" t="inlineStr">
         <is>
-          <t>page 169-189; Abstract: households spending &gt;3% of income on water acquisition, DHA vulnerability</t>
+          <t>page 169-189; Method (formulas for average household water spending and the 3% criterion); section on water in Hid</t>
         </is>
       </c>
       <c r="G519" s="2" t="inlineStr">
@@ -26022,7 +26022,7 @@
       </c>
       <c r="I519" s="2" t="inlineStr">
         <is>
-          <t>Hidalgo has the largest number of wastewater discharge points for agricultural purposes in Mexico, and scarce sectoral regulation combined with gradual contamination of rivers/streams is identified as a risk factor for increasing the number of under-supplied households. Households in Hidalgo were found to be vulnerable under the Human Right to Water (DHA) framework, spending more than 3% of income</t>
+          <t>In 2020, 96% of the population of Hidalgo had piped water (66.9% inside the dwelling, 29.1% within the plot; 80% from the public service and 15.7% from community wells) and 94% sewerage; coverage is lowest in Huautla (65.2%), La Misión (68.4%), Yahualica (72.8%) and Tepehuacán (75.3%); 50.8% of the population is poor and 11.8% indigenous; water pressure is medium-strong (32.3%). With one minimum s</t>
         </is>
       </c>
       <c r="J519" s="2" t="inlineStr"/>
@@ -26057,7 +26057,7 @@
       </c>
       <c r="F520" s="2" t="inlineStr">
         <is>
-          <t>page 169-189; Abstract: households spending &gt;3% of income on water acquisition, DHA vulnerability</t>
+          <t>page 169-189; Method (formulas for average household water spending and the 3% criterion); section on water in Hid</t>
         </is>
       </c>
       <c r="G520" s="2" t="inlineStr">
@@ -26107,7 +26107,7 @@
       </c>
       <c r="F521" s="2" t="inlineStr">
         <is>
-          <t>page 169-189; Abstract: households spending &gt;3% of income on water acquisition, DHA vulnerability</t>
+          <t>page 169-189; Method (formulas for average household water spending and the 3% criterion); section on water in Hid</t>
         </is>
       </c>
       <c r="G521" s="2" t="inlineStr">
@@ -26157,7 +26157,7 @@
       </c>
       <c r="F522" s="2" t="inlineStr">
         <is>
-          <t>page 169-189; Abstract: households spending &gt;3% of income on water acquisition, DHA vulnerability</t>
+          <t>page 169-189; Method (formulas for average household water spending and the 3% criterion); section on water in Hid</t>
         </is>
       </c>
       <c r="G522" s="2" t="inlineStr">
@@ -26207,7 +26207,7 @@
       </c>
       <c r="F523" s="2" t="inlineStr">
         <is>
-          <t>page 169-189; Abstract: households spending &gt;3% of income on water acquisition, DHA vulnerability</t>
+          <t>page 169-189; Method (formulas for average household water spending and the 3% criterion); section on water in Hid</t>
         </is>
       </c>
       <c r="G523" s="2" t="inlineStr">

</xml_diff>